<commit_message>
updated time frame of growth expectation
</commit_message>
<xml_diff>
--- a/decision_matrix.xlsx
+++ b/decision_matrix.xlsx
@@ -1,19 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://habselstree-my.sharepoint.com/personal/agupte14167_habselstree_org_uk/Documents/Year 12/ERP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F00C03D4-68EF-1840-8DBD-2926AD015544}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="135" documentId="8_{F00C03D4-68EF-1840-8DBD-2926AD015544}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5A2AFDF6-7A1B-A84B-B995-A5AAA7189BC7}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28420" windowHeight="16940" xr2:uid="{ACF530BF-67BC-054D-9ADF-0FF83347B423}"/>
+    <workbookView xWindow="14620" yWindow="500" windowWidth="14180" windowHeight="17500" xr2:uid="{ACF530BF-67BC-054D-9ADF-0FF83347B423}"/>
   </bookViews>
   <sheets>
     <sheet name="Inputs" sheetId="1" r:id="rId1"/>
+    <sheet name="Provider_Scores" sheetId="3" r:id="rId2"/>
+    <sheet name="Deployment_Scores" sheetId="4" r:id="rId3"/>
+    <sheet name="Service_Scores" sheetId="5" r:id="rId4"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -36,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="44">
   <si>
     <t>Input Name</t>
   </si>
@@ -104,10 +107,70 @@
     <t>0 &lt;= X &lt;= 100</t>
   </si>
   <si>
-    <t>Growth expectation (give time frame)</t>
-  </si>
-  <si>
     <t>Integer – estimated growth multiplier</t>
+  </si>
+  <si>
+    <t>Criterion</t>
+  </si>
+  <si>
+    <t>Cost</t>
+  </si>
+  <si>
+    <t>Scalability</t>
+  </si>
+  <si>
+    <t>Sustainability</t>
+  </si>
+  <si>
+    <t>AWS</t>
+  </si>
+  <si>
+    <t>Azure</t>
+  </si>
+  <si>
+    <t>Google Cloud</t>
+  </si>
+  <si>
+    <t>Cost (monthly, per GB)</t>
+  </si>
+  <si>
+    <t>Geographic coverage</t>
+  </si>
+  <si>
+    <t>Security</t>
+  </si>
+  <si>
+    <t>Public</t>
+  </si>
+  <si>
+    <t>Private</t>
+  </si>
+  <si>
+    <t>Hybrid</t>
+  </si>
+  <si>
+    <t>Multicloud</t>
+  </si>
+  <si>
+    <t>Technical Complexity</t>
+  </si>
+  <si>
+    <t>IaaS</t>
+  </si>
+  <si>
+    <t>PaaS</t>
+  </si>
+  <si>
+    <t>SaaS</t>
+  </si>
+  <si>
+    <t>Customisability</t>
+  </si>
+  <si>
+    <t>Management Overhead</t>
+  </si>
+  <si>
+    <t>Growth expectation (5 year time frame)</t>
   </si>
 </sst>
 </file>
@@ -156,7 +219,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -164,6 +227,14 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -604,16 +675,325 @@
     </row>
     <row r="8" spans="1:4" ht="51" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>22</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>23</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B0CE183-3D9A-8341-BEA7-54599B6C5049}">
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="20.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="40" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2" s="6">
+        <v>8</v>
+      </c>
+      <c r="C2" s="6">
+        <v>5</v>
+      </c>
+      <c r="D2" s="6">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" s="6">
+        <v>9</v>
+      </c>
+      <c r="C3" s="6">
+        <v>9</v>
+      </c>
+      <c r="D3" s="6">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" s="6">
+        <v>7</v>
+      </c>
+      <c r="C4" s="6">
+        <v>7</v>
+      </c>
+      <c r="D4" s="6">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" s="6">
+        <v>9</v>
+      </c>
+      <c r="C5" s="6">
+        <v>9</v>
+      </c>
+      <c r="D5" s="6">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" s="6">
+        <v>9</v>
+      </c>
+      <c r="C6" s="6">
+        <v>9</v>
+      </c>
+      <c r="D6" s="6">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4D49A44-0E36-034E-963D-AA4E1BC5CD0C}">
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="19.1640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" s="6">
+        <v>8</v>
+      </c>
+      <c r="C2" s="6">
+        <v>3</v>
+      </c>
+      <c r="D2" s="6">
+        <v>5</v>
+      </c>
+      <c r="E2" s="6">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" s="6">
+        <v>9</v>
+      </c>
+      <c r="C3" s="6">
+        <v>4</v>
+      </c>
+      <c r="D3" s="6">
+        <v>5</v>
+      </c>
+      <c r="E3" s="6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="6">
+        <v>9</v>
+      </c>
+      <c r="C4" s="6">
+        <v>5</v>
+      </c>
+      <c r="D4" s="6">
+        <v>8</v>
+      </c>
+      <c r="E4" s="6">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="6">
+        <v>7</v>
+      </c>
+      <c r="C5" s="6">
+        <v>5</v>
+      </c>
+      <c r="D5" s="6">
+        <v>7</v>
+      </c>
+      <c r="E5" s="6">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" s="6">
+        <v>5</v>
+      </c>
+      <c r="C6" s="6">
+        <v>10</v>
+      </c>
+      <c r="D6" s="6">
+        <v>8</v>
+      </c>
+      <c r="E6" s="6">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86295259-9A01-6448-A06F-16C523E941B9}">
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="20.1640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" s="6">
+        <v>7</v>
+      </c>
+      <c r="C2" s="6">
+        <v>6</v>
+      </c>
+      <c r="D2" s="6">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" s="6">
+        <v>3</v>
+      </c>
+      <c r="C3" s="6">
+        <v>6</v>
+      </c>
+      <c r="D3" s="6">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" s="6">
+        <v>6</v>
+      </c>
+      <c r="C4" s="6">
+        <v>7</v>
+      </c>
+      <c r="D4" s="6">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B5" s="6">
+        <v>10</v>
+      </c>
+      <c r="C5" s="6">
+        <v>7</v>
+      </c>
+      <c r="D5" s="6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" s="6">
+        <v>3</v>
+      </c>
+      <c r="C6" s="6">
+        <v>6</v>
+      </c>
+      <c r="D6" s="6">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>